<commit_message>
modified:   examples/Accrection/A_Embryos_Composition.ipynb 	modified:   examples/Accrection/Tables/note_02_early_composition.csv 	modified:   examples/Cosmochemistry/Tables/A1_IW35IW15_composition.csv 	modified:   examples/Impact/Tables/note_02_giant_impact.xlsx 	modified:   examples/Impact/Tables/note_02_small_impact.xlsx 	modified:   examples/quickstart/03_Embryo_bulk_composition.ipynb 	modified:   src/accrediff/__init__.py 	modified:   src/accrediff/chemistry.py 	modified:   src/accrediff/differentiation.py 	modified:   src/accrediff/gas_migration.py 	modified:   src/accrediff/plotting.py
</commit_message>
<xml_diff>
--- a/examples/Impact/Tables/note_02_giant_impact.xlsx
+++ b/examples/Impact/Tables/note_02_giant_impact.xlsx
@@ -4890,10 +4890,10 @@
         </is>
       </c>
       <c r="I127" t="n">
-        <v>91.65268779916667</v>
+        <v>51.77158917206075</v>
       </c>
       <c r="J127" t="n">
-        <v>4119.326177868897</v>
+        <v>3360.170310036875</v>
       </c>
       <c r="K127" t="n">
         <v>1</v>
@@ -4927,10 +4927,10 @@
         </is>
       </c>
       <c r="I128" t="n">
-        <v>40.77453455974334</v>
+        <v>39.51288432207557</v>
       </c>
       <c r="J128" t="n">
-        <v>3043.196860944978</v>
+        <v>3002.969250708737</v>
       </c>
       <c r="K128" t="n">
         <v>1</v>
@@ -4964,10 +4964,10 @@
         </is>
       </c>
       <c r="I129" t="n">
-        <v>40.77453455974334</v>
+        <v>39.51288432207557</v>
       </c>
       <c r="J129" t="n">
-        <v>3043.196860944978</v>
+        <v>3002.969250708737</v>
       </c>
       <c r="K129" t="n">
         <v>1</v>
@@ -8012,13 +8012,13 @@
         </is>
       </c>
       <c r="I72" t="n">
-        <v>10.99747999186293</v>
+        <v>5.542247559988567</v>
       </c>
       <c r="J72" t="n">
-        <v>2298.817419929961</v>
+        <v>2131.04566118994</v>
       </c>
       <c r="K72" t="n">
-        <v>0.4221056819434598</v>
+        <v>0.4013600545969349</v>
       </c>
     </row>
     <row r="73">
@@ -8049,13 +8049,13 @@
         </is>
       </c>
       <c r="I73" t="n">
-        <v>3.939443745638553</v>
+        <v>3.62767617576676</v>
       </c>
       <c r="J73" t="n">
-        <v>2066.539874888375</v>
+        <v>2053.105019131273</v>
       </c>
       <c r="K73" t="n">
-        <v>0.4221056819434598</v>
+        <v>0.4013600545969349</v>
       </c>
     </row>
     <row r="74">
@@ -8121,13 +8121,13 @@
         </is>
       </c>
       <c r="I75" t="n">
-        <v>3.939443745638553</v>
+        <v>3.62767617576676</v>
       </c>
       <c r="J75" t="n">
-        <v>2066.539874888375</v>
+        <v>2053.105019131273</v>
       </c>
       <c r="K75" t="n">
-        <v>0.4221056819434598</v>
+        <v>0.4013600545969349</v>
       </c>
     </row>
     <row r="76">
@@ -8193,13 +8193,13 @@
         </is>
       </c>
       <c r="I77" t="n">
-        <v>3.939443745638553</v>
+        <v>3.62767617576676</v>
       </c>
       <c r="J77" t="n">
-        <v>2066.539874888375</v>
+        <v>2053.105019131273</v>
       </c>
       <c r="K77" t="n">
-        <v>0.4221056819434598</v>
+        <v>0.4013600545969349</v>
       </c>
     </row>
     <row r="78">
@@ -8265,13 +8265,13 @@
         </is>
       </c>
       <c r="I79" t="n">
-        <v>3.939443745638553</v>
+        <v>3.62767617576676</v>
       </c>
       <c r="J79" t="n">
-        <v>2066.539874888375</v>
+        <v>2053.105019131273</v>
       </c>
       <c r="K79" t="n">
-        <v>0.4221056819434598</v>
+        <v>0.4013600545969349</v>
       </c>
     </row>
     <row r="80">
@@ -8302,13 +8302,13 @@
         </is>
       </c>
       <c r="I80" t="n">
-        <v>3.939443745638553</v>
+        <v>3.62767617576676</v>
       </c>
       <c r="J80" t="n">
-        <v>2066.539874888375</v>
+        <v>2053.105019131273</v>
       </c>
       <c r="K80" t="n">
-        <v>0.4221056819434598</v>
+        <v>0.4013600545969349</v>
       </c>
     </row>
     <row r="81">
@@ -8374,13 +8374,13 @@
         </is>
       </c>
       <c r="I82" t="n">
-        <v>3.939443745638553</v>
+        <v>3.62767617576676</v>
       </c>
       <c r="J82" t="n">
-        <v>2066.539874888375</v>
+        <v>2053.105019131273</v>
       </c>
       <c r="K82" t="n">
-        <v>0.4221056819434598</v>
+        <v>0.4013600545969349</v>
       </c>
     </row>
     <row r="83">
@@ -8656,13 +8656,13 @@
         </is>
       </c>
       <c r="I90" t="n">
-        <v>10.33712423779653</v>
+        <v>5.112434655994025</v>
       </c>
       <c r="J90" t="n">
-        <v>2282.375610999227</v>
+        <v>2114.482829993046</v>
       </c>
       <c r="K90" t="n">
-        <v>0.3492843298509574</v>
+        <v>0.3320817721422925</v>
       </c>
     </row>
     <row r="91">
@@ -8728,13 +8728,13 @@
         </is>
       </c>
       <c r="I92" t="n">
-        <v>3.793499197272463</v>
+        <v>3.465947014264299</v>
       </c>
       <c r="J92" t="n">
-        <v>2060.287557314621</v>
+        <v>2046.01875945332</v>
       </c>
       <c r="K92" t="n">
-        <v>0.3492843298509574</v>
+        <v>0.3320817721422925</v>
       </c>
     </row>
     <row r="93">
@@ -8765,13 +8765,13 @@
         </is>
       </c>
       <c r="I93" t="n">
-        <v>3.793499197272463</v>
+        <v>3.465947014264299</v>
       </c>
       <c r="J93" t="n">
-        <v>2060.287557314621</v>
+        <v>2046.01875945332</v>
       </c>
       <c r="K93" t="n">
-        <v>0.3492843298509574</v>
+        <v>0.3320817721422925</v>
       </c>
     </row>
     <row r="94">
@@ -8837,13 +8837,13 @@
         </is>
       </c>
       <c r="I95" t="n">
-        <v>50.91350282734524</v>
+        <v>28.38170055329934</v>
       </c>
       <c r="J95" t="n">
-        <v>3337.500887854836</v>
+        <v>2610.053001450451</v>
       </c>
       <c r="K95" t="n">
-        <v>0.9478574529434155</v>
+        <v>0.900897651513955</v>
       </c>
     </row>
     <row r="96">
@@ -8874,13 +8874,13 @@
         </is>
       </c>
       <c r="I96" t="n">
-        <v>19.33602544032931</v>
+        <v>16.80858534322889</v>
       </c>
       <c r="J96" t="n">
-        <v>2434.768637377907</v>
+        <v>2405.754092195194</v>
       </c>
       <c r="K96" t="n">
-        <v>0.9478574529434155</v>
+        <v>0.900897651513955</v>
       </c>
     </row>
     <row r="97">

</xml_diff>